<commit_message>
floodfill method and its findings
</commit_message>
<xml_diff>
--- a/pathfinding_recordings.xlsx
+++ b/pathfinding_recordings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asmis\Documents\COMPSYS301_team2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B54BB8-F766-4D89-8287-E6B0C8C33FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77599F85-7738-4697-9E3A-9F78BCE3F05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{7700CBF5-08F8-4E5E-A6C4-5AD761BAA852}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="17">
   <si>
     <t>algorithm</t>
   </si>
@@ -85,6 +85,12 @@
   </si>
   <si>
     <t>GBF</t>
+  </si>
+  <si>
+    <t>floodfill</t>
+  </si>
+  <si>
+    <t>[14,8]</t>
   </si>
 </sst>
 </file>
@@ -456,7 +462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CCF085A-D1B2-4377-B6BE-870B791A9AB1}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -650,6 +656,42 @@
         <v>8</v>
       </c>
       <c r="D16">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19">
         <v>77</v>
       </c>
     </row>
@@ -660,7 +702,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC9C14E6-257F-483B-AFD0-26ADBB495A4C}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -857,6 +899,42 @@
         <v>26</v>
       </c>
     </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>